<commit_message>
Update AI main insights - אנליסט
</commit_message>
<xml_diff>
--- a/ai_main_insights.xlsx
+++ b/ai_main_insights.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,47 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>אנליסט</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>מה יש כרגע על הפרק?</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>**פרויקט "אנליסט" - עדכון סטטוס ומצב נוכחי**
+נכון להיום, פרויקט "אנליסט" נמצא בסטטוס **אדום** ומוגדר כפרויקט **אקטיבי**.
+**מצב משימות ולוחות זמנים:**
+*   **"העלאת גרסה בעמיתים לטסט"** הושלמה בהצלחה על ידי אלישבע שליסל, עם יעד תאריך של 2026-05-14.
+*   **"בדיקת גרסת עמיתים בטסטים"** נמצאת בביצוע, באחריותה של ורד גדנקן, ויעד התאריך לסיומה הוא 2026-05-17.
+*   **"העלאת גרסת עמיתים לייצור"** ממתינה לאישור הלקוח, באחריות אלישבע שליסל, עם יעד תאריך של 2026-05-19.
+*   **"הגדרת פתרון מאובטח לבעיית גישה בייצור"** ממתינה לאישור אבט"מ, באחריות מתן שרון, עם יעד תאריך של 2026-05-20.
+**סיכונים רלוונטיים:**
+*   **חוסר רציפות בפיתוח — תנודתיות עומס:** סיכון בעל הסתברות והשפעה גבוהות (4/5, 4/5) בקטגוריית משאבים. מציין כי חוסר עבודה רציפה ומלאה בפיתוח, ועומס לא צפוי, מובילים לאי-עמידה בלוחות זמנים.
+*   **עיכובים בגלל תלות בעיצוב וניתוח:** סיכון בעל הסתברות גבוהה (4/5) והשפעה בינונית (3/5) בקטגוריית לוח זמנים. הסיבה היא שבקשות הדורשות עיצוב/ניתוח מעכבות דליברי, מכיוון שמשאבים אלו מוקצים לפרויקטים אחרים.
+*   **אי-עמידה ב-SLA העלאת גרסה חודשית:** סיכון בעל הסתברות בינונית (3/5) והשפעה גבוהה (4/5) בקטגוריית לוח זמנים. הלקוח מצפה לעדכון גרסה חודשי.
+*   **מערכת מעסיקים — קוד ישן וקשיח לשינויים:** סיכון בעל הסתברות והשפעה גבוהות (4/5, 4/5) בקטגוריה הטכנית. מערכת זו ישנה, והשינויים בה מסוכנים ויקרים.
+**משאבי צוות פעילים:**
+*   **סיון פרידמן:** מנהלת פרויקטים, 25% העסקה.
+*   **אלישבע שליסל:** מפתחת Backend, 33% העסקה.
+*   **ורד גדנקן:** מנהלת בדיקות, 10% העסקה.
+**💡 תובנות והמלצות**
+*   **התמודדות עם חוסר רציפות בפיתוח:** יש לבחון מחדש את הקצאת המשאבים על מנת להבטיח זרימת עבודה רציפה יותר בפרויקט "אנליסט" ולהימנע מעומסים לא צפויים.
+*   **שיפור יעילות תלויות חיצוניות:** מומלץ לבחון אפיקים לקיצור זמני ההמתנה לעיצוב וניתוח, או להקצאת משאבים ייעודיים לפתרון תלויות אלו, על מנת למנוע עיכובים בלוחות הזמנים.
+*   **עדכון תהליכי שחרור גרסאות:** יש לוודא שהתהליכים הנוכחיים עומדים בדרישת הלקוח להעלאת גרסה חודשית, ולבחון דרכים לייעל את תהליך השחרור על מנת לעמוד ב-SLA.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>17/05/2026 20:05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update AI main insights - דלק
</commit_message>
<xml_diff>
--- a/ai_main_insights.xlsx
+++ b/ai_main_insights.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -528,6 +528,58 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>דלק</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">מהם הסיכונים כרגע בפרויקט? </t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>להלן סקירה של הסיכונים הקיימים בפרויקט "דלק":
+**סיכונים פתוחים:**
+*   **תלות קריטית במפתחת יחידה — אין גיבוי ידע:**
+    *   **הסתברות:** 5/5
+    *   **השפעה:** 5/5
+    *   **קטגוריה:** משאבים
+    *   **הערות:** סיכון קריטי הנובע מכך שרק מפתחת אחת מכירה את המערכת מקצה לקצה.
+*   **עומס לא צפוי — מפתחת בפרויקט אחר במקביל:**
+    *   **הסתברות:** 4/5
+    *   **השפעה:** 4/5
+    *   **קטגוריה:** לוח זמנים
+    *   **הערות:** המפתחת כבר מחויבת למשימות בפרויקט אחר, מה שעלול להוביל לעיכובים כאשר משימות חדשות מגיעות.
+*   **הזמנות עבודה לא מתחדשות בזמן:**
+    *   **הסתברות:** 4/5
+    *   **השפעה:** 4/5
+    *   **קטגוריה:** תקציב
+    *   **הערות:** קיים צורך לתזכר את הלקוח כל חודשיים, ויש סיכון להפסקת כיסוי כספי.
+*   **קשר חלש מול הלקוח — חוסר נראות:**
+    *   **הסתברות:** 3/5
+    *   **השפעה:** 3/5
+    *   **קטגוריה:** חיצוני
+    *   **הערות:** חוסר בתמונה מלאה של הנעשה אצל הלקוח מעבר למשימות שנפתחות.
+*   **תלות בממשקי ליבה של הלקוח:**
+    *   **הסתברות:** 3/5
+    *   **השפעה:** 4/5
+    *   **קטגוריה:** טכני
+    *   **הערות:** שינויים במערכות הליבה של הלקוח עלולים להשפיע באופן מהותי וקריטי על המערכת שלנו.
+**💡 תובנות והמלצות**
+*   **טיפול מיידי בתלות במפתחת יחידה:** יש לפתח תוכנית לגיבוי ידע והכשרת משאב נוסף למערכת, על מנת להפחית את הסיכון הקריטי.
+*   **תיאום עומסים וסדרי עדיפויות:** יש לבצע תיאום מול הלקוח לגבי עומסים עתידיים ולבחון אפשרויות לסדר עדיפויות בין הפרויקטים בהם המפתחת מעורבת.
+*   **חיזוק הקשר מול הלקוח:** יש ליזום פגישות תכופות יותר עם הלקוח ולהגדיר מנגנוני דיווח שוטפים, על מנת לשפר את הנראות ולהפחית את הסיכון לתקשורת לקויה.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>17/05/2026 20:22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>